<commit_message>
Git commit prior to merge
</commit_message>
<xml_diff>
--- a/artifacts/api-server/src/python/phase16_exports/Validation_Report.xlsx
+++ b/artifacts/api-server/src/python/phase16_exports/Validation_Report.xlsx
@@ -439,7 +439,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -490,8 +490,10 @@
           <t>win_rate_pct</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>66.7</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -500,8 +502,10 @@
           <t>profit_factor</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>8.75</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -510,8 +514,10 @@
           <t>expectancy</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>155</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -520,8 +526,10 @@
           <t>max_drawdown_pct</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>1.15</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -530,8 +538,10 @@
           <t>sharpe_ratio</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>13.05</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -540,8 +550,10 @@
           <t>avg_holding_days</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>0</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -550,8 +562,10 @@
           <t>avg_risk_reward</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>2.6</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -571,7 +585,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5465</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="16">
@@ -581,7 +595,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9.300000000000001</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -663,50 +677,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AI Scan</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>SBIN (300.0)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ICICIBANK (-60.0)</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Watch</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Only 3 trades — keep collecting evidence (need 5+).</t>
-        </is>
-      </c>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -859,22 +843,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>50</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -884,22 +874,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F6" t="n">
-        <v>7.35</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -913,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1021,254 +1017,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.848369</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.851094</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1020</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1095</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H2" t="n">
-        <v>7.35</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>82</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>AI Scan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Near target — partial exit</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>AI engine APPROVES the BUY signal for SBIN. RR 3.2:1 with full 4/4 timeframe agreement and BULLISH regime. Confidence 82/100.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Setup conditions repeated here are worth prioritising.</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>High entry confidence (82.0); Favourable risk/reward (3.2:1); Exit discipline: target hit as planned</t>
-        </is>
-      </c>
+          <t>No completed trades yet</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.836435</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.838630</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1380</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-60</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-1.43</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LOW_VOLATILITY</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>65</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>AI Scan</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Stop loss triggered</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>AI engine approved ICICIBANK signal. RR 2.1:1, 3/4 timeframes agree. Confidence 65/100.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Review whether the entry matched the regime and quality gates.</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Stop-loss hit — entry timing or stop placement to review</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.831728</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-07-08T21:50:57.833771</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>820</v>
-      </c>
-      <c r="E4" t="n">
-        <v>865</v>
-      </c>
-      <c r="F4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" t="n">
-        <v>225</v>
-      </c>
-      <c r="H4" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LOW_VOLATILITY</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>72</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>AI Scan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Target approached — taking profit</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>AI engine approved HDFCBANK BUY. RR 2.5:1 with 3/4 timeframe agreement. LOW_VOLATILITY regime supports breakout entries. Confidence adjusted to 72/100.</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Setup conditions repeated here are worth prioritising.</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>High entry confidence (72.0); Favourable risk/reward (2.5:1); Exit discipline: target hit as planned</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1324,7 +1094,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Insufficient Data — only 3 completed trades; need 5+ per strategy/regime cell before recommendations become meaningful.</t>
+          <t>Insufficient Data — only 0 completed trades; need 5+ per strategy/regime cell before recommendations become meaningful.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>